<commit_message>
fixed tests for new convolve with smaller output images, except morphology that doesn't combine images of different sizes
</commit_message>
<xml_diff>
--- a/src/test/transform-image-create/sample_gray.xlsx
+++ b/src/test/transform-image-create/sample_gray.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kushn\Dropbox\software\projects\cv\local\cv-workbench\src\test\transform-image-create\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kushn\Dropbox\software\projects\cv\cv-workbench\src\test\transform-image-create\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C11007A3-9B2A-4053-9AED-014265F77E9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5ED9EA8-C220-4EFF-9BBC-DCC7D043A049}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8920" yWindow="3450" windowWidth="12170" windowHeight="7980" activeTab="1" xr2:uid="{38C2D0CF-08BD-45AE-9870-6D0409E0CC5E}"/>
+    <workbookView xWindow="3396" yWindow="792" windowWidth="19572" windowHeight="11880" activeTab="1" xr2:uid="{38C2D0CF-08BD-45AE-9870-6D0409E0CC5E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,6 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="25">
   <si>
     <t>rows</t>
   </si>
@@ -55,19 +54,98 @@
   </si>
   <si>
     <t>max_col</t>
+  </si>
+  <si>
+    <t>src_rows</t>
+  </si>
+  <si>
+    <t>src_cols</t>
+  </si>
+  <si>
+    <t>out_cols</t>
+  </si>
+  <si>
+    <t>out_rows</t>
+  </si>
+  <si>
+    <t>src_min_row</t>
+  </si>
+  <si>
+    <t>src_min_col</t>
+  </si>
+  <si>
+    <t>row</t>
+  </si>
+  <si>
+    <t>0..5</t>
+  </si>
+  <si>
+    <t>col</t>
+  </si>
+  <si>
+    <t>0..6</t>
+  </si>
+  <si>
+    <t>=</t>
+  </si>
+  <si>
+    <t>3..10</t>
+  </si>
+  <si>
+    <t>3,2-10,8</t>
+  </si>
+  <si>
+    <t>8x7</t>
+  </si>
+  <si>
+    <t>out</t>
+  </si>
+  <si>
+    <t>6x7</t>
+  </si>
+  <si>
+    <t>image_header</t>
+  </si>
+  <si>
+    <t>min_row</t>
+  </si>
+  <si>
+    <t>min_col</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="0.0"/>
+  </numFmts>
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1" tint="4.9989318521683403E-2"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10.5"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="10.5"/>
+      <color theme="1"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="4">
@@ -90,7 +168,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -178,11 +256,150 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="dashed">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="dashed">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="dashed">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="dashed">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="dashed">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="dashed">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -194,18 +411,41 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -521,18 +761,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B36994EF-DA8C-4682-9C92-D2CC3B0525EC}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="8.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.7265625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -540,7 +780,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -548,7 +788,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -562,7 +802,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4">
       <c r="A4">
         <v>0</v>
       </c>
@@ -578,7 +818,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4">
       <c r="A5">
         <v>4</v>
       </c>
@@ -594,7 +834,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4">
       <c r="A6">
         <v>5</v>
       </c>
@@ -610,7 +850,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4">
       <c r="A7">
         <v>6</v>
       </c>
@@ -633,32 +873,34 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDAEE9BB-117D-4078-B93B-BD6340D85A31}">
-  <dimension ref="A1:S15"/>
-  <sheetFormatPr defaultColWidth="6.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:AB26"/>
+  <sheetFormatPr defaultColWidth="6.6640625" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="12" width="4.6328125" customWidth="1"/>
+    <col min="1" max="12" width="4.6640625" customWidth="1"/>
+    <col min="14" max="20" width="6.77734375" customWidth="1"/>
+    <col min="21" max="21" width="8.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28">
       <c r="B1">
         <v>0</v>
       </c>
-      <c r="C1" s="20">
+      <c r="C1" s="11">
         <v>1</v>
       </c>
-      <c r="D1" s="20">
+      <c r="D1" s="11">
         <v>2</v>
       </c>
-      <c r="E1" s="20">
+      <c r="E1" s="11">
         <v>3</v>
       </c>
-      <c r="F1" s="20">
+      <c r="F1" s="11">
         <v>4</v>
       </c>
-      <c r="G1" s="20">
+      <c r="G1" s="11">
         <v>5</v>
       </c>
-      <c r="H1" s="20">
+      <c r="H1" s="11">
         <v>6</v>
       </c>
       <c r="I1">
@@ -674,7 +916,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:28">
       <c r="A2">
         <v>0</v>
       </c>
@@ -711,30 +953,39 @@
       <c r="L2" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A3" s="20">
+      <c r="N2" t="s">
+        <v>18</v>
+      </c>
+      <c r="P2" s="26" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:28">
+      <c r="A3" s="11">
         <v>1</v>
       </c>
       <c r="B3" s="4">
         <v>0</v>
       </c>
-      <c r="C3" s="12">
-        <v>0</v>
-      </c>
-      <c r="D3" s="15">
-        <v>0</v>
-      </c>
-      <c r="E3" s="15">
-        <v>0</v>
-      </c>
-      <c r="F3" s="15">
-        <v>0</v>
-      </c>
-      <c r="G3" s="15">
-        <v>0</v>
-      </c>
-      <c r="H3" s="16">
+      <c r="C3" s="5">
+        <v>0</v>
+      </c>
+      <c r="D3" s="5">
+        <v>0</v>
+      </c>
+      <c r="E3" s="5">
+        <v>0</v>
+      </c>
+      <c r="F3" s="5">
+        <v>0</v>
+      </c>
+      <c r="G3" s="5">
+        <v>0</v>
+      </c>
+      <c r="H3" s="5">
         <v>0</v>
       </c>
       <c r="I3" s="5">
@@ -749,282 +1000,319 @@
       <c r="L3" s="6">
         <v>0</v>
       </c>
-      <c r="N3">
-        <v>0</v>
-      </c>
-      <c r="O3" s="20">
+      <c r="P3" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" ht="15" thickBot="1">
+      <c r="A4" s="11">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5">
+        <v>0</v>
+      </c>
+      <c r="D4" s="7">
+        <v>255</v>
+      </c>
+      <c r="E4" s="7">
+        <v>255</v>
+      </c>
+      <c r="F4" s="7">
+        <v>255</v>
+      </c>
+      <c r="G4" s="5">
+        <v>0</v>
+      </c>
+      <c r="H4" s="12">
+        <v>0</v>
+      </c>
+      <c r="I4" s="5">
+        <v>0</v>
+      </c>
+      <c r="J4" s="7">
+        <v>255</v>
+      </c>
+      <c r="K4" s="5">
+        <v>0</v>
+      </c>
+      <c r="L4" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28">
+      <c r="A5" s="11">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5">
+        <v>0</v>
+      </c>
+      <c r="D5" s="13">
+        <v>255</v>
+      </c>
+      <c r="E5" s="14">
+        <v>255</v>
+      </c>
+      <c r="F5" s="14">
+        <v>255</v>
+      </c>
+      <c r="G5" s="15">
+        <v>0</v>
+      </c>
+      <c r="H5" s="15">
+        <v>0</v>
+      </c>
+      <c r="I5" s="15">
+        <v>0</v>
+      </c>
+      <c r="J5" s="16">
+        <v>255</v>
+      </c>
+      <c r="K5" s="5">
+        <v>0</v>
+      </c>
+      <c r="L5" s="6">
+        <v>0</v>
+      </c>
+      <c r="N5" s="11">
+        <v>0</v>
+      </c>
+      <c r="O5" s="11">
         <v>1</v>
       </c>
-      <c r="P3" s="20">
+      <c r="P5" s="11">
         <v>2</v>
       </c>
-      <c r="Q3" s="20">
+      <c r="Q5" s="11">
         <v>3</v>
       </c>
-      <c r="R3" s="20">
+      <c r="R5" s="11">
         <v>4</v>
       </c>
-      <c r="S3" s="20">
+      <c r="S5" s="11">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A4" s="20">
-        <v>2</v>
-      </c>
-      <c r="B4" s="4">
-        <v>0</v>
-      </c>
-      <c r="C4" s="13">
-        <v>0</v>
-      </c>
-      <c r="D4" s="7">
-        <v>255</v>
-      </c>
-      <c r="E4" s="7">
-        <v>255</v>
-      </c>
-      <c r="F4" s="7">
-        <v>255</v>
-      </c>
-      <c r="G4" s="5">
-        <v>0</v>
-      </c>
-      <c r="H4" s="17">
-        <v>0</v>
-      </c>
-      <c r="I4" s="5">
-        <v>0</v>
-      </c>
-      <c r="J4" s="7">
-        <v>255</v>
-      </c>
-      <c r="K4" s="5">
-        <v>0</v>
-      </c>
-      <c r="L4" s="6">
-        <v>0</v>
-      </c>
-      <c r="M4">
-        <v>0</v>
-      </c>
-      <c r="N4" s="22">
-        <f>D3*0.25+D4*0.5+D5*0.25</f>
+      <c r="T5" s="11">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28">
+      <c r="A6" s="11">
+        <v>4</v>
+      </c>
+      <c r="B6" s="4">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5">
+        <v>0</v>
+      </c>
+      <c r="D6" s="31">
+        <v>255</v>
+      </c>
+      <c r="E6" s="32">
+        <v>255</v>
+      </c>
+      <c r="F6" s="32">
+        <v>255</v>
+      </c>
+      <c r="G6" s="33">
+        <v>0</v>
+      </c>
+      <c r="H6" s="33">
+        <v>0</v>
+      </c>
+      <c r="I6" s="33">
+        <v>0</v>
+      </c>
+      <c r="J6" s="34">
+        <v>255</v>
+      </c>
+      <c r="K6" s="5">
+        <v>0</v>
+      </c>
+      <c r="L6" s="6">
+        <v>0</v>
+      </c>
+      <c r="M6" s="11">
+        <v>0</v>
+      </c>
+      <c r="N6" s="39">
+        <f>D5*0.25+D6*0.5+D7*0.25</f>
+        <v>255</v>
+      </c>
+      <c r="O6" s="39">
+        <f t="shared" ref="O6:O11" si="0">E5*0.25+E6*0.5+E7*0.25</f>
+        <v>255</v>
+      </c>
+      <c r="P6" s="39">
+        <f t="shared" ref="P6:P11" si="1">F5*0.25+F6*0.5+F7*0.25</f>
+        <v>255</v>
+      </c>
+      <c r="Q6" s="39">
+        <f t="shared" ref="Q6:Q11" si="2">G5*0.25+G6*0.5+G7*0.25</f>
+        <v>0</v>
+      </c>
+      <c r="R6" s="39">
+        <f t="shared" ref="R6:R11" si="3">H5*0.25+H6*0.5+H7*0.25</f>
+        <v>0</v>
+      </c>
+      <c r="S6" s="39">
+        <f t="shared" ref="S6:S11" si="4">I5*0.25+I6*0.5+I7*0.25</f>
+        <v>0</v>
+      </c>
+      <c r="T6" s="39">
+        <f t="shared" ref="T6:T11" si="5">J5*0.25+J6*0.5+J7*0.25</f>
+        <v>255</v>
+      </c>
+      <c r="V6">
+        <v>255</v>
+      </c>
+      <c r="W6">
+        <v>255</v>
+      </c>
+      <c r="X6">
+        <v>255</v>
+      </c>
+      <c r="Y6">
+        <v>0</v>
+      </c>
+      <c r="Z6">
+        <v>0</v>
+      </c>
+      <c r="AA6">
+        <v>0</v>
+      </c>
+      <c r="AB6">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28">
+      <c r="A7" s="11">
+        <v>5</v>
+      </c>
+      <c r="B7" s="4">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5">
+        <v>0</v>
+      </c>
+      <c r="D7" s="27">
+        <v>255</v>
+      </c>
+      <c r="E7" s="17">
+        <v>255</v>
+      </c>
+      <c r="F7" s="17">
+        <v>255</v>
+      </c>
+      <c r="G7" s="18">
+        <v>0</v>
+      </c>
+      <c r="H7" s="18">
+        <v>0</v>
+      </c>
+      <c r="I7" s="18">
+        <v>0</v>
+      </c>
+      <c r="J7" s="28">
+        <v>255</v>
+      </c>
+      <c r="K7" s="5">
+        <v>0</v>
+      </c>
+      <c r="L7" s="6">
+        <v>0</v>
+      </c>
+      <c r="M7" s="11">
+        <v>1</v>
+      </c>
+      <c r="N7" s="39">
+        <f t="shared" ref="N7:N11" si="6">D6*0.25+D7*0.5+D8*0.25</f>
         <v>191.25</v>
       </c>
-      <c r="O4" s="22">
-        <f t="shared" ref="O4:O11" si="0">E3*0.25+E4*0.5+E5*0.25</f>
-        <v>191.25</v>
-      </c>
-      <c r="P4" s="22">
-        <f t="shared" ref="P4:P11" si="1">F3*0.25+F4*0.5+F5*0.25</f>
-        <v>191.25</v>
-      </c>
-      <c r="Q4" s="21">
-        <f t="shared" ref="Q4:Q11" si="2">G3*0.25+G4*0.5+G5*0.25</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A5" s="20">
-        <v>3</v>
-      </c>
-      <c r="B5" s="4">
-        <v>0</v>
-      </c>
-      <c r="C5" s="13">
-        <v>0</v>
-      </c>
-      <c r="D5" s="7">
-        <v>255</v>
-      </c>
-      <c r="E5" s="7">
-        <v>255</v>
-      </c>
-      <c r="F5" s="7">
-        <v>255</v>
-      </c>
-      <c r="G5" s="5">
-        <v>0</v>
-      </c>
-      <c r="H5" s="17">
-        <v>0</v>
-      </c>
-      <c r="I5" s="5">
-        <v>0</v>
-      </c>
-      <c r="J5" s="7">
-        <v>255</v>
-      </c>
-      <c r="K5" s="5">
-        <v>0</v>
-      </c>
-      <c r="L5" s="6">
-        <v>0</v>
-      </c>
-      <c r="M5" s="20">
-        <v>1</v>
-      </c>
-      <c r="N5" s="22">
-        <f t="shared" ref="N5:N11" si="3">D4*0.25+D5*0.5+D6*0.25</f>
-        <v>255</v>
-      </c>
-      <c r="O5" s="22">
-        <f t="shared" si="0"/>
-        <v>255</v>
-      </c>
-      <c r="P5" s="22">
-        <f t="shared" si="1"/>
-        <v>255</v>
-      </c>
-      <c r="Q5" s="21">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A6" s="20">
-        <v>4</v>
-      </c>
-      <c r="B6" s="4">
-        <v>0</v>
-      </c>
-      <c r="C6" s="13">
-        <v>0</v>
-      </c>
-      <c r="D6" s="7">
-        <v>255</v>
-      </c>
-      <c r="E6" s="7">
-        <v>255</v>
-      </c>
-      <c r="F6" s="7">
-        <v>255</v>
-      </c>
-      <c r="G6" s="5">
-        <v>0</v>
-      </c>
-      <c r="H6" s="17">
-        <v>0</v>
-      </c>
-      <c r="I6" s="5">
-        <v>0</v>
-      </c>
-      <c r="J6" s="7">
-        <v>255</v>
-      </c>
-      <c r="K6" s="5">
-        <v>0</v>
-      </c>
-      <c r="L6" s="6">
-        <v>0</v>
-      </c>
-      <c r="M6" s="20">
-        <v>2</v>
-      </c>
-      <c r="N6" s="22">
-        <f t="shared" si="3"/>
-        <v>255</v>
-      </c>
-      <c r="O6" s="22">
-        <f t="shared" si="0"/>
-        <v>255</v>
-      </c>
-      <c r="P6" s="22">
-        <f t="shared" si="1"/>
-        <v>255</v>
-      </c>
-      <c r="Q6" s="21">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A7" s="20">
-        <v>5</v>
-      </c>
-      <c r="B7" s="4">
-        <v>0</v>
-      </c>
-      <c r="C7" s="13">
-        <v>0</v>
-      </c>
-      <c r="D7" s="7">
-        <v>255</v>
-      </c>
-      <c r="E7" s="7">
-        <v>255</v>
-      </c>
-      <c r="F7" s="7">
-        <v>255</v>
-      </c>
-      <c r="G7" s="5">
-        <v>0</v>
-      </c>
-      <c r="H7" s="17">
-        <v>0</v>
-      </c>
-      <c r="I7" s="5">
-        <v>0</v>
-      </c>
-      <c r="J7" s="7">
-        <v>255</v>
-      </c>
-      <c r="K7" s="5">
-        <v>0</v>
-      </c>
-      <c r="L7" s="6">
-        <v>0</v>
-      </c>
-      <c r="M7" s="20">
-        <v>3</v>
-      </c>
-      <c r="N7" s="22">
-        <f t="shared" si="3"/>
-        <v>191.25</v>
-      </c>
-      <c r="O7" s="22">
+      <c r="O7" s="39">
         <f t="shared" si="0"/>
         <v>191.25</v>
       </c>
-      <c r="P7" s="22">
+      <c r="P7" s="39">
         <f t="shared" si="1"/>
         <v>191.25</v>
       </c>
-      <c r="Q7" s="21">
+      <c r="Q7" s="39">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A8" s="20">
+      <c r="R7" s="39">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="S7" s="39">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="T7" s="39">
+        <f t="shared" si="5"/>
+        <v>255</v>
+      </c>
+      <c r="V7">
+        <v>191.25</v>
+      </c>
+      <c r="W7">
+        <v>191.25</v>
+      </c>
+      <c r="X7">
+        <v>191.25</v>
+      </c>
+      <c r="Y7">
+        <v>0</v>
+      </c>
+      <c r="Z7">
+        <v>0</v>
+      </c>
+      <c r="AA7">
+        <v>0</v>
+      </c>
+      <c r="AB7">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28">
+      <c r="A8" s="11">
         <v>6</v>
       </c>
       <c r="B8" s="4">
         <v>0</v>
       </c>
-      <c r="C8" s="13">
-        <v>0</v>
-      </c>
-      <c r="D8" s="5">
-        <v>0</v>
-      </c>
-      <c r="E8" s="5">
-        <v>0</v>
-      </c>
-      <c r="F8" s="5">
-        <v>0</v>
-      </c>
-      <c r="G8" s="5">
-        <v>0</v>
-      </c>
-      <c r="H8" s="17">
-        <v>0</v>
-      </c>
-      <c r="I8" s="5">
-        <v>0</v>
-      </c>
-      <c r="J8" s="7">
+      <c r="C8" s="5">
+        <v>0</v>
+      </c>
+      <c r="D8" s="29">
+        <v>0</v>
+      </c>
+      <c r="E8" s="18">
+        <v>0</v>
+      </c>
+      <c r="F8" s="18">
+        <v>0</v>
+      </c>
+      <c r="G8" s="18">
+        <v>0</v>
+      </c>
+      <c r="H8" s="18">
+        <v>0</v>
+      </c>
+      <c r="I8" s="18">
+        <v>0</v>
+      </c>
+      <c r="J8" s="28">
         <v>255</v>
       </c>
       <c r="K8" s="5">
@@ -1033,55 +1321,88 @@
       <c r="L8" s="6">
         <v>0</v>
       </c>
-      <c r="M8" s="20">
-        <v>4</v>
-      </c>
-      <c r="N8" s="22">
-        <f t="shared" si="3"/>
+      <c r="M8" s="11">
+        <v>2</v>
+      </c>
+      <c r="N8" s="39">
+        <f t="shared" si="6"/>
         <v>63.75</v>
       </c>
-      <c r="O8" s="22">
+      <c r="O8" s="39">
         <f t="shared" si="0"/>
         <v>63.75</v>
       </c>
-      <c r="P8" s="22">
+      <c r="P8" s="39">
         <f t="shared" si="1"/>
         <v>63.75</v>
       </c>
-      <c r="Q8" s="21">
+      <c r="Q8" s="39">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A9" s="20">
+      <c r="R8" s="39">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="S8" s="39">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="T8" s="39">
+        <f t="shared" si="5"/>
+        <v>255</v>
+      </c>
+      <c r="V8">
+        <v>63.75</v>
+      </c>
+      <c r="W8">
+        <v>63.75</v>
+      </c>
+      <c r="X8">
+        <v>63.75</v>
+      </c>
+      <c r="Y8">
+        <v>0</v>
+      </c>
+      <c r="Z8">
+        <v>0</v>
+      </c>
+      <c r="AA8">
+        <v>0</v>
+      </c>
+      <c r="AB8">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28">
+      <c r="A9" s="11">
         <v>7</v>
       </c>
       <c r="B9" s="4">
         <v>0</v>
       </c>
-      <c r="C9" s="13">
-        <v>0</v>
-      </c>
-      <c r="D9" s="5">
-        <v>0</v>
-      </c>
-      <c r="E9" s="5">
-        <v>0</v>
-      </c>
-      <c r="F9" s="5">
-        <v>0</v>
-      </c>
-      <c r="G9" s="5">
-        <v>0</v>
-      </c>
-      <c r="H9" s="17">
-        <v>0</v>
-      </c>
-      <c r="I9" s="5">
-        <v>0</v>
-      </c>
-      <c r="J9" s="7">
+      <c r="C9" s="5">
+        <v>0</v>
+      </c>
+      <c r="D9" s="29">
+        <v>0</v>
+      </c>
+      <c r="E9" s="18">
+        <v>0</v>
+      </c>
+      <c r="F9" s="18">
+        <v>0</v>
+      </c>
+      <c r="G9" s="18">
+        <v>0</v>
+      </c>
+      <c r="H9" s="18">
+        <v>0</v>
+      </c>
+      <c r="I9" s="18">
+        <v>0</v>
+      </c>
+      <c r="J9" s="28">
         <v>255</v>
       </c>
       <c r="K9" s="5">
@@ -1090,55 +1411,88 @@
       <c r="L9" s="6">
         <v>0</v>
       </c>
-      <c r="M9" s="20">
-        <v>5</v>
-      </c>
-      <c r="N9" s="22">
-        <f t="shared" si="3"/>
+      <c r="M9" s="11">
+        <v>3</v>
+      </c>
+      <c r="N9" s="39">
+        <f t="shared" si="6"/>
         <v>63.75</v>
       </c>
-      <c r="O9" s="22">
+      <c r="O9" s="39">
         <f t="shared" si="0"/>
         <v>63.75</v>
       </c>
-      <c r="P9" s="22">
+      <c r="P9" s="39">
         <f t="shared" si="1"/>
         <v>63.75</v>
       </c>
-      <c r="Q9" s="21">
+      <c r="Q9" s="39">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A10" s="20">
+      <c r="R9" s="39">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="S9" s="39">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="T9" s="39">
+        <f t="shared" si="5"/>
+        <v>191.25</v>
+      </c>
+      <c r="V9">
+        <v>63.75</v>
+      </c>
+      <c r="W9">
+        <v>63.75</v>
+      </c>
+      <c r="X9">
+        <v>63.75</v>
+      </c>
+      <c r="Y9">
+        <v>0</v>
+      </c>
+      <c r="Z9">
+        <v>0</v>
+      </c>
+      <c r="AA9">
+        <v>0</v>
+      </c>
+      <c r="AB9">
+        <v>191.25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28">
+      <c r="A10" s="11">
         <v>8</v>
       </c>
       <c r="B10" s="4">
         <v>0</v>
       </c>
-      <c r="C10" s="13">
-        <v>0</v>
-      </c>
-      <c r="D10" s="7">
-        <v>255</v>
-      </c>
-      <c r="E10" s="7">
-        <v>255</v>
-      </c>
-      <c r="F10" s="7">
-        <v>255</v>
-      </c>
-      <c r="G10" s="5">
-        <v>0</v>
-      </c>
-      <c r="H10" s="17">
-        <v>0</v>
-      </c>
-      <c r="I10" s="5">
-        <v>0</v>
-      </c>
-      <c r="J10" s="5">
+      <c r="C10" s="5">
+        <v>0</v>
+      </c>
+      <c r="D10" s="27">
+        <v>255</v>
+      </c>
+      <c r="E10" s="17">
+        <v>255</v>
+      </c>
+      <c r="F10" s="17">
+        <v>255</v>
+      </c>
+      <c r="G10" s="18">
+        <v>0</v>
+      </c>
+      <c r="H10" s="18">
+        <v>0</v>
+      </c>
+      <c r="I10" s="18">
+        <v>0</v>
+      </c>
+      <c r="J10" s="30">
         <v>0</v>
       </c>
       <c r="K10" s="5">
@@ -1147,55 +1501,88 @@
       <c r="L10" s="6">
         <v>0</v>
       </c>
-      <c r="M10" s="20">
-        <v>6</v>
-      </c>
-      <c r="N10" s="22">
-        <f t="shared" si="3"/>
+      <c r="M10" s="11">
+        <v>4</v>
+      </c>
+      <c r="N10" s="39">
+        <f t="shared" si="6"/>
         <v>191.25</v>
       </c>
-      <c r="O10" s="22">
+      <c r="O10" s="39">
         <f t="shared" si="0"/>
         <v>127.5</v>
       </c>
-      <c r="P10" s="22">
+      <c r="P10" s="39">
         <f t="shared" si="1"/>
         <v>191.25</v>
       </c>
-      <c r="Q10" s="21">
+      <c r="Q10" s="39">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A11" s="20">
+      <c r="R10" s="39">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="S10" s="39">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="T10" s="39">
+        <f t="shared" si="5"/>
+        <v>63.75</v>
+      </c>
+      <c r="V10">
+        <v>191.25</v>
+      </c>
+      <c r="W10">
+        <v>127.5</v>
+      </c>
+      <c r="X10">
+        <v>191.25</v>
+      </c>
+      <c r="Y10">
+        <v>0</v>
+      </c>
+      <c r="Z10">
+        <v>0</v>
+      </c>
+      <c r="AA10">
+        <v>0</v>
+      </c>
+      <c r="AB10">
+        <v>63.75</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28">
+      <c r="A11" s="11">
         <v>9</v>
       </c>
       <c r="B11" s="4">
         <v>0</v>
       </c>
-      <c r="C11" s="13">
-        <v>0</v>
-      </c>
-      <c r="D11" s="7">
-        <v>255</v>
-      </c>
-      <c r="E11" s="5">
-        <v>0</v>
-      </c>
-      <c r="F11" s="7">
-        <v>255</v>
-      </c>
-      <c r="G11" s="5">
-        <v>0</v>
-      </c>
-      <c r="H11" s="17">
-        <v>0</v>
-      </c>
-      <c r="I11" s="5">
-        <v>0</v>
-      </c>
-      <c r="J11" s="5">
+      <c r="C11" s="5">
+        <v>0</v>
+      </c>
+      <c r="D11" s="35">
+        <v>255</v>
+      </c>
+      <c r="E11" s="36">
+        <v>0</v>
+      </c>
+      <c r="F11" s="37">
+        <v>255</v>
+      </c>
+      <c r="G11" s="36">
+        <v>0</v>
+      </c>
+      <c r="H11" s="36">
+        <v>0</v>
+      </c>
+      <c r="I11" s="36">
+        <v>0</v>
+      </c>
+      <c r="J11" s="38">
         <v>0</v>
       </c>
       <c r="K11" s="5">
@@ -1204,55 +1591,88 @@
       <c r="L11" s="6">
         <v>0</v>
       </c>
-      <c r="M11" s="20">
-        <v>7</v>
-      </c>
-      <c r="N11" s="22">
-        <f t="shared" si="3"/>
-        <v>255</v>
-      </c>
-      <c r="O11" s="22">
+      <c r="M11" s="11">
+        <v>5</v>
+      </c>
+      <c r="N11" s="39">
+        <f t="shared" si="6"/>
+        <v>255</v>
+      </c>
+      <c r="O11" s="39">
         <f t="shared" si="0"/>
         <v>63.75</v>
       </c>
-      <c r="P11" s="22">
+      <c r="P11" s="39">
         <f t="shared" si="1"/>
         <v>255</v>
       </c>
-      <c r="Q11" s="21">
+      <c r="Q11" s="39">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A12" s="20">
+      <c r="R11" s="39">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="S11" s="39">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="T11" s="39">
+        <f t="shared" si="5"/>
+        <v>63.75</v>
+      </c>
+      <c r="V11">
+        <v>255</v>
+      </c>
+      <c r="W11">
+        <v>63.75</v>
+      </c>
+      <c r="X11">
+        <v>255</v>
+      </c>
+      <c r="Y11">
+        <v>0</v>
+      </c>
+      <c r="Z11">
+        <v>0</v>
+      </c>
+      <c r="AA11">
+        <v>0</v>
+      </c>
+      <c r="AB11">
+        <v>63.75</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28" ht="15" thickBot="1">
+      <c r="A12" s="11">
         <v>10</v>
       </c>
       <c r="B12" s="4">
         <v>0</v>
       </c>
-      <c r="C12" s="14">
-        <v>0</v>
-      </c>
-      <c r="D12" s="11">
-        <v>255</v>
-      </c>
-      <c r="E12" s="19">
-        <v>0</v>
-      </c>
-      <c r="F12" s="11">
-        <v>255</v>
-      </c>
-      <c r="G12" s="19">
-        <v>0</v>
-      </c>
-      <c r="H12" s="18">
-        <v>0</v>
-      </c>
-      <c r="I12" s="5">
-        <v>0</v>
-      </c>
-      <c r="J12" s="7">
+      <c r="C12" s="5">
+        <v>0</v>
+      </c>
+      <c r="D12" s="19">
+        <v>255</v>
+      </c>
+      <c r="E12" s="20">
+        <v>0</v>
+      </c>
+      <c r="F12" s="21">
+        <v>255</v>
+      </c>
+      <c r="G12" s="20">
+        <v>0</v>
+      </c>
+      <c r="H12" s="20">
+        <v>0</v>
+      </c>
+      <c r="I12" s="20">
+        <v>0</v>
+      </c>
+      <c r="J12" s="22">
         <v>255</v>
       </c>
       <c r="K12" s="5">
@@ -1262,7 +1682,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:28">
       <c r="A13">
         <v>11</v>
       </c>
@@ -1299,8 +1719,23 @@
       <c r="L13" s="6">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="W13">
+        <v>0</v>
+      </c>
+      <c r="X13">
+        <v>-255</v>
+      </c>
+      <c r="Y13">
+        <v>-255</v>
+      </c>
+      <c r="Z13">
+        <v>0</v>
+      </c>
+      <c r="AA13">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="14" spans="1:28">
       <c r="A14">
         <v>12</v>
       </c>
@@ -1337,8 +1772,23 @@
       <c r="L14" s="6">
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="W14">
+        <v>0</v>
+      </c>
+      <c r="X14">
+        <v>-191.25</v>
+      </c>
+      <c r="Y14">
+        <v>-191.25</v>
+      </c>
+      <c r="Z14">
+        <v>0</v>
+      </c>
+      <c r="AA14">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="15" spans="1:28">
       <c r="A15">
         <v>13</v>
       </c>
@@ -1374,6 +1824,354 @@
       </c>
       <c r="L15" s="10">
         <v>0</v>
+      </c>
+      <c r="W15">
+        <v>0</v>
+      </c>
+      <c r="X15">
+        <v>-63.75</v>
+      </c>
+      <c r="Y15">
+        <v>-63.75</v>
+      </c>
+      <c r="Z15">
+        <v>0</v>
+      </c>
+      <c r="AA15">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="16" spans="1:28">
+      <c r="W16">
+        <v>0</v>
+      </c>
+      <c r="X16">
+        <v>-63.75</v>
+      </c>
+      <c r="Y16">
+        <v>-63.75</v>
+      </c>
+      <c r="Z16">
+        <v>0</v>
+      </c>
+      <c r="AA16">
+        <v>191.25</v>
+      </c>
+    </row>
+    <row r="17" spans="2:27">
+      <c r="P17" t="s">
+        <v>22</v>
+      </c>
+      <c r="W17">
+        <v>0</v>
+      </c>
+      <c r="X17">
+        <v>-127.5</v>
+      </c>
+      <c r="Y17">
+        <v>-191.25</v>
+      </c>
+      <c r="Z17">
+        <v>0</v>
+      </c>
+      <c r="AA17">
+        <v>63.75</v>
+      </c>
+    </row>
+    <row r="18" spans="2:27">
+      <c r="B18" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="3">
+        <v>8</v>
+      </c>
+      <c r="J18" t="s">
+        <v>12</v>
+      </c>
+      <c r="L18" t="s">
+        <v>13</v>
+      </c>
+      <c r="N18" s="26" t="s">
+        <v>16</v>
+      </c>
+      <c r="O18" t="s">
+        <v>17</v>
+      </c>
+      <c r="P18" t="s">
+        <v>0</v>
+      </c>
+      <c r="R18">
+        <v>14</v>
+      </c>
+      <c r="W18">
+        <v>0</v>
+      </c>
+      <c r="X18">
+        <v>-63.75</v>
+      </c>
+      <c r="Y18">
+        <v>-255</v>
+      </c>
+      <c r="Z18">
+        <v>0</v>
+      </c>
+      <c r="AA18">
+        <v>63.75</v>
+      </c>
+    </row>
+    <row r="19" spans="2:27">
+      <c r="B19" s="25" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="10">
+        <v>7</v>
+      </c>
+      <c r="K19" t="s">
+        <v>14</v>
+      </c>
+      <c r="M19" t="s">
+        <v>15</v>
+      </c>
+      <c r="P19" t="s">
+        <v>1</v>
+      </c>
+      <c r="R19">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" spans="2:27">
+      <c r="B20" s="24" t="s">
+        <v>0</v>
+      </c>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="3">
+        <v>3</v>
+      </c>
+      <c r="P20" t="s">
+        <v>23</v>
+      </c>
+      <c r="R20">
+        <v>3</v>
+      </c>
+      <c r="T20" t="s">
+        <v>0</v>
+      </c>
+      <c r="U20">
+        <f>R22-R20+1</f>
+        <v>8</v>
+      </c>
+      <c r="W20">
+        <f>X6-V6</f>
+        <v>0</v>
+      </c>
+      <c r="X20">
+        <f t="shared" ref="X20:AA20" si="7">Y6-W6</f>
+        <v>-255</v>
+      </c>
+      <c r="Y20">
+        <f t="shared" si="7"/>
+        <v>-255</v>
+      </c>
+      <c r="Z20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="AA20">
+        <f t="shared" si="7"/>
+        <v>255</v>
+      </c>
+    </row>
+    <row r="21" spans="2:27">
+      <c r="B21" s="25" t="s">
+        <v>1</v>
+      </c>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="10">
+        <v>1</v>
+      </c>
+      <c r="P21" t="s">
+        <v>24</v>
+      </c>
+      <c r="R21">
+        <v>2</v>
+      </c>
+      <c r="T21" t="s">
+        <v>1</v>
+      </c>
+      <c r="U21">
+        <f>R23-R21+1</f>
+        <v>7</v>
+      </c>
+      <c r="W21">
+        <f t="shared" ref="W21:AA21" si="8">X7-V7</f>
+        <v>0</v>
+      </c>
+      <c r="X21">
+        <f t="shared" si="8"/>
+        <v>-191.25</v>
+      </c>
+      <c r="Y21">
+        <f t="shared" si="8"/>
+        <v>-191.25</v>
+      </c>
+      <c r="Z21">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="AA21">
+        <f t="shared" si="8"/>
+        <v>255</v>
+      </c>
+    </row>
+    <row r="22" spans="2:27">
+      <c r="B22" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
+      <c r="F22" s="3">
+        <v>6</v>
+      </c>
+      <c r="P22" t="s">
+        <v>4</v>
+      </c>
+      <c r="R22">
+        <v>10</v>
+      </c>
+      <c r="W22">
+        <f t="shared" ref="W22:AA22" si="9">X8-V8</f>
+        <v>0</v>
+      </c>
+      <c r="X22">
+        <f t="shared" si="9"/>
+        <v>-63.75</v>
+      </c>
+      <c r="Y22">
+        <f t="shared" si="9"/>
+        <v>-63.75</v>
+      </c>
+      <c r="Z22">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="AA22">
+        <f t="shared" si="9"/>
+        <v>255</v>
+      </c>
+    </row>
+    <row r="23" spans="2:27">
+      <c r="B23" s="25" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23" s="9"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="10">
+        <v>7</v>
+      </c>
+      <c r="P23" t="s">
+        <v>5</v>
+      </c>
+      <c r="R23">
+        <v>8</v>
+      </c>
+      <c r="W23">
+        <f t="shared" ref="W23:AA23" si="10">X9-V9</f>
+        <v>0</v>
+      </c>
+      <c r="X23">
+        <f t="shared" si="10"/>
+        <v>-63.75</v>
+      </c>
+      <c r="Y23">
+        <f t="shared" si="10"/>
+        <v>-63.75</v>
+      </c>
+      <c r="Z23">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="AA23">
+        <f t="shared" si="10"/>
+        <v>191.25</v>
+      </c>
+    </row>
+    <row r="24" spans="2:27">
+      <c r="B24" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="3">
+        <v>3</v>
+      </c>
+      <c r="W24">
+        <f t="shared" ref="W24:AA24" si="11">X10-V10</f>
+        <v>0</v>
+      </c>
+      <c r="X24">
+        <f t="shared" si="11"/>
+        <v>-127.5</v>
+      </c>
+      <c r="Y24">
+        <f t="shared" si="11"/>
+        <v>-191.25</v>
+      </c>
+      <c r="Z24">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="AA24">
+        <f t="shared" si="11"/>
+        <v>63.75</v>
+      </c>
+    </row>
+    <row r="25" spans="2:27">
+      <c r="B25" s="25" t="s">
+        <v>11</v>
+      </c>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="10">
+        <v>2</v>
+      </c>
+      <c r="W25">
+        <f t="shared" ref="W25:AA25" si="12">X11-V11</f>
+        <v>0</v>
+      </c>
+      <c r="X25">
+        <f t="shared" si="12"/>
+        <v>-63.75</v>
+      </c>
+      <c r="Y25">
+        <f t="shared" si="12"/>
+        <v>-255</v>
+      </c>
+      <c r="Z25">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="AA25">
+        <f t="shared" si="12"/>
+        <v>63.75</v>
+      </c>
+    </row>
+    <row r="26" spans="2:27">
+      <c r="B26" s="23" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>